<commit_message>
Fix Lessons i18n and prevent student group race condition
</commit_message>
<xml_diff>
--- a/TTOptimizer.Web/Data/Nauczyciele.xlsx
+++ b/TTOptimizer.Web/Data/Nauczyciele.xlsx
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
-  <si>
-    <t xml:space="preserve">Name</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
   <si>
     <t xml:space="preserve">Apolonia Wysocka</t>
   </si>
@@ -169,6 +166,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -228,8 +226,12 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -356,235 +358,230 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A44"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="45.63"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.96"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>30</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+      <c r="A38" s="1" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="1" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="A40" s="1" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="A41" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="A42" s="1" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
+      <c r="A43" s="1" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+      <c r="A44" s="1" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
-        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: streamline class generation and lesson setup
</commit_message>
<xml_diff>
--- a/TTOptimizer.Web/Data/Nauczyciele.xlsx
+++ b/TTOptimizer.Web/Data/Nauczyciele.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">Apolonia Wysocka</t>
   </si>
@@ -71,87 +71,6 @@
   </si>
   <si>
     <t xml:space="preserve">Roksana Gajda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Seweryn Jurewicz</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tamara Bieńkowska</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ulryk Pawlik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Wiktoria Cichoń</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zbigniew Rosiak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aurelia Michalak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Borys Kaczmarek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Daria Łuczak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Eryk Mielczarek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Felicja Kubera</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gniewomir Baran</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Honorata Frączek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Idzi Rogalski</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jowita Dąbek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kajetan Musiał</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lidia Żmuda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Maksymilian Olejnik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nina Kołodziej</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Olgierd Czarnecki</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Polina Lisowska</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Radosław Kulesza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sabina Tomczak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Teodor Niziołek</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Urszula Janik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Witold Chmiel</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Żaneta Woźniak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mirosław Płonka</t>
   </si>
 </sst>
 </file>
@@ -358,7 +277,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A44"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27.96"/>
@@ -447,141 +366,6 @@
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
         <v>16</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="1" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="1" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="s">
-        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>